<commit_message>
Regenerate project files (#532)
</commit_message>
<xml_diff>
--- a/project/excel/sssom_schema.xlsx
+++ b/project/excel/sssom_schema.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV1"/>
+  <dimension ref="A1:AX1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -817,70 +817,80 @@
       </c>
       <c r="AI1" t="inlineStr">
         <is>
+          <t>review_date</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
           <t>confidence</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>reviewer_agreement</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
         <is>
           <t>curation_rule</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>curation_rule_text</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>subject_match_field</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>object_match_field</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>match_string</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>subject_preprocessing</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>object_preprocessing</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>similarity_score</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AT1" t="inlineStr">
         <is>
           <t>similarity_measure</t>
         </is>
       </c>
-      <c r="AS1" t="inlineStr">
+      <c r="AU1" t="inlineStr">
         <is>
           <t>see_also</t>
         </is>
       </c>
-      <c r="AT1" t="inlineStr">
+      <c r="AV1" t="inlineStr">
         <is>
           <t>issue_tracker_item</t>
         </is>
       </c>
-      <c r="AU1" t="inlineStr">
+      <c r="AW1" t="inlineStr">
         <is>
           <t>other</t>
         </is>
       </c>
-      <c r="AV1" t="inlineStr">
+      <c r="AX1" t="inlineStr">
         <is>
           <t>comment</t>
         </is>

</xml_diff>

<commit_message>
Rebuild project after adding `derives_from` slot to Mapping model (#549)
Following #538, this PR rebuilds all artifacts with `make gen-project`
</commit_message>
<xml_diff>
--- a/project/excel/sssom_schema.xlsx
+++ b/project/excel/sssom_schema.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX1"/>
+  <dimension ref="A1:AY1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -887,10 +887,15 @@
       </c>
       <c r="AW1" t="inlineStr">
         <is>
+          <t>derived_from</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
           <t>other</t>
         </is>
       </c>
-      <c r="AX1" t="inlineStr">
+      <c r="AY1" t="inlineStr">
         <is>
           <t>comment</t>
         </is>

</xml_diff>